<commit_message>
Update training_log.xlsx from TRAINING05
</commit_message>
<xml_diff>
--- a/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
+++ b/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
@@ -11,6 +11,7 @@
     <sheet name="testTask" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="test2" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="test3" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="test1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3975,4 +3976,979 @@
   </sheetData>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AY14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col customWidth="1" max="1" min="1" width="14"/>
+    <col customWidth="1" max="2" min="2" width="14"/>
+    <col customWidth="1" max="3" min="3" width="14"/>
+    <col customWidth="1" max="4" min="4" width="14"/>
+    <col customWidth="1" max="5" min="5" width="14"/>
+    <col customWidth="1" max="6" min="6" width="14"/>
+    <col customWidth="1" max="7" min="7" width="14"/>
+    <col customWidth="1" max="8" min="8" width="14"/>
+    <col customWidth="1" max="9" min="9" width="14"/>
+    <col customWidth="1" max="10" min="10" width="14"/>
+    <col customWidth="1" max="11" min="11" width="14"/>
+    <col customWidth="1" max="12" min="12" width="14"/>
+    <col customWidth="1" max="13" min="13" width="14"/>
+    <col customWidth="1" max="14" min="14" width="14"/>
+    <col customWidth="1" max="15" min="15" width="14"/>
+    <col customWidth="1" max="16" min="16" width="14"/>
+    <col customWidth="1" max="17" min="17" width="14"/>
+    <col customWidth="1" max="18" min="18" width="14"/>
+    <col customWidth="1" max="19" min="19" width="14"/>
+    <col customWidth="1" max="20" min="20" width="14"/>
+    <col customWidth="1" max="21" min="21" width="14"/>
+    <col customWidth="1" max="22" min="22" width="14"/>
+    <col customWidth="1" max="23" min="23" width="14"/>
+    <col customWidth="1" max="24" min="24" width="14"/>
+    <col customWidth="1" max="25" min="25" width="14"/>
+    <col customWidth="1" max="26" min="26" width="14"/>
+    <col customWidth="1" max="27" min="27" width="14"/>
+    <col customWidth="1" max="28" min="28" width="14"/>
+    <col customWidth="1" max="29" min="29" width="14"/>
+    <col customWidth="1" max="30" min="30" width="14"/>
+    <col customWidth="1" max="31" min="31" width="14"/>
+    <col customWidth="1" max="32" min="32" width="14"/>
+    <col customWidth="1" max="33" min="33" width="14"/>
+    <col customWidth="1" max="34" min="34" width="14"/>
+    <col customWidth="1" max="35" min="35" width="14"/>
+    <col customWidth="1" max="36" min="36" width="14"/>
+    <col customWidth="1" max="37" min="37" width="14"/>
+    <col customWidth="1" max="38" min="38" width="14"/>
+    <col customWidth="1" max="39" min="39" width="14"/>
+    <col customWidth="1" max="40" min="40" width="14"/>
+    <col customWidth="1" max="41" min="41" width="14"/>
+    <col customWidth="1" max="42" min="42" width="14"/>
+    <col customWidth="1" max="43" min="43" width="14"/>
+    <col customWidth="1" max="44" min="44" width="14"/>
+    <col customWidth="1" max="45" min="45" width="14"/>
+    <col customWidth="1" max="46" min="46" width="14"/>
+    <col customWidth="1" max="47" min="47" width="14"/>
+    <col customWidth="1" max="48" min="48" width="14"/>
+    <col customWidth="1" hidden="1" max="49" min="49" width="14"/>
+    <col customWidth="1" max="50" min="50" width="14"/>
+    <col customWidth="1" max="51" min="51" width="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Animal: test1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>DOB</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Sex</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Strain</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Baseline weight (g)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Time (HH:MM)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Weight (g)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Weight %</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Weight after task (g)</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Weight after task %</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Water given by hand after task</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Trials</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Duration (s)</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Reward Amount (uL)</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Total Volume (uL)</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>Aborts</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>Withheld</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>No-movement</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+      <c r="P7" s="3" t="inlineStr">
+        <is>
+          <t>Wheel Aborts</t>
+        </is>
+      </c>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>L turns</t>
+        </is>
+      </c>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>R turns</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>Licks</t>
+        </is>
+      </c>
+      <c r="T7" s="3" t="inlineStr">
+        <is>
+          <t>Threshold start (deg)</t>
+        </is>
+      </c>
+      <c r="U7" s="3" t="inlineStr">
+        <is>
+          <t>Threshold end (deg)</t>
+        </is>
+      </c>
+      <c r="V7" s="3" t="inlineStr">
+        <is>
+          <t>Threshold end (% final)</t>
+        </is>
+      </c>
+      <c r="W7" s="3" t="inlineStr">
+        <is>
+          <t>ITI (s)</t>
+        </is>
+      </c>
+      <c r="X7" s="3" t="inlineStr">
+        <is>
+          <t>Gain mult (Stage 1)</t>
+        </is>
+      </c>
+      <c r="Y7" s="3" t="inlineStr">
+        <is>
+          <t>Direction ratio (Stage 2)</t>
+        </is>
+      </c>
+      <c r="Z7" s="3" t="inlineStr">
+        <is>
+          <t>Simple gates met</t>
+        </is>
+      </c>
+      <c r="AA7" s="3" t="inlineStr">
+        <is>
+          <t>Response Thresh Start (deg)</t>
+        </is>
+      </c>
+      <c r="AB7" s="3" t="inlineStr">
+        <is>
+          <t>Response Thresh End (deg)</t>
+        </is>
+      </c>
+      <c r="AC7" s="3" t="inlineStr">
+        <is>
+          <t>Quiescence Start (s)</t>
+        </is>
+      </c>
+      <c r="AD7" s="3" t="inlineStr">
+        <is>
+          <t>Quiescence End (s)</t>
+        </is>
+      </c>
+      <c r="AE7" s="3" t="inlineStr">
+        <is>
+          <t>In-trial Threshold (deg)</t>
+        </is>
+      </c>
+      <c r="AF7" s="3" t="inlineStr">
+        <is>
+          <t>Click Attenuated (Stage 4)</t>
+        </is>
+      </c>
+      <c r="AG7" s="3" t="inlineStr">
+        <is>
+          <t>Accuracy (gamma=1.0)</t>
+        </is>
+      </c>
+      <c r="AH7" s="3" t="inlineStr">
+        <is>
+          <t>Abort Rate</t>
+        </is>
+      </c>
+      <c r="AI7" s="3" t="inlineStr">
+        <is>
+          <t>Aborts: Quiescence</t>
+        </is>
+      </c>
+      <c r="AJ7" s="3" t="inlineStr">
+        <is>
+          <t>Aborts: Cue</t>
+        </is>
+      </c>
+      <c r="AK7" s="3" t="inlineStr">
+        <is>
+          <t>Aborts: Delay</t>
+        </is>
+      </c>
+      <c r="AL7" s="3" t="inlineStr">
+        <is>
+          <t>Aborts: Response</t>
+        </is>
+      </c>
+      <c r="AM7" s="3" t="inlineStr">
+        <is>
+          <t>Warmup Trials</t>
+        </is>
+      </c>
+      <c r="AN7" s="3" t="inlineStr">
+        <is>
+          <t>Repeat Trials</t>
+        </is>
+      </c>
+      <c r="AO7" s="3" t="inlineStr">
+        <is>
+          <t>Session Water (uL)</t>
+        </is>
+      </c>
+      <c r="AP7" s="3" t="inlineStr">
+        <is>
+          <t>Staircase Advanced (Stage 5)</t>
+        </is>
+      </c>
+      <c r="AQ7" s="3" t="inlineStr">
+        <is>
+          <t>Git Commit</t>
+        </is>
+      </c>
+      <c r="AR7" s="3" t="inlineStr">
+        <is>
+          <t>Target SPL (dB)</t>
+        </is>
+      </c>
+      <c r="AS7" s="3" t="inlineStr">
+        <is>
+          <t>Left Freq (Hz)</t>
+        </is>
+      </c>
+      <c r="AT7" s="3" t="inlineStr">
+        <is>
+          <t>Right Freq (Hz)</t>
+        </is>
+      </c>
+      <c r="AU7" s="3" t="inlineStr">
+        <is>
+          <t>Num. Sessions</t>
+        </is>
+      </c>
+      <c r="AV7" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="AW7" s="3" t="inlineStr">
+        <is>
+          <t>Session started</t>
+        </is>
+      </c>
+      <c r="AX7" s="3" t="inlineStr">
+        <is>
+          <t>Session data (local path)</t>
+        </is>
+      </c>
+      <c r="AY7" s="3" t="inlineStr">
+        <is>
+          <t>Session struct (local path)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="7" t="n"/>
+      <c r="J8" s="7" t="n"/>
+      <c r="K8" s="7" t="n"/>
+      <c r="L8" s="7" t="n"/>
+      <c r="M8" s="7" t="n"/>
+      <c r="N8" s="7" t="n"/>
+      <c r="O8" s="7" t="n"/>
+      <c r="P8" s="7" t="n"/>
+      <c r="Q8" s="7" t="n"/>
+      <c r="R8" s="7" t="n"/>
+      <c r="S8" s="7" t="n"/>
+      <c r="T8" s="7" t="n"/>
+      <c r="U8" s="7" t="n"/>
+      <c r="V8" s="7" t="n"/>
+      <c r="W8" s="7" t="n"/>
+      <c r="X8" s="7" t="n"/>
+      <c r="Y8" s="7" t="n"/>
+      <c r="Z8" s="7" t="n"/>
+      <c r="AA8" s="7" t="n"/>
+      <c r="AB8" s="7" t="n"/>
+      <c r="AC8" s="7" t="n"/>
+      <c r="AD8" s="7" t="n"/>
+      <c r="AE8" s="7" t="n"/>
+      <c r="AF8" s="7" t="n"/>
+      <c r="AG8" s="7" t="n"/>
+      <c r="AH8" s="7" t="n"/>
+      <c r="AI8" s="7" t="n"/>
+      <c r="AJ8" s="7" t="n"/>
+      <c r="AK8" s="7" t="n"/>
+      <c r="AL8" s="7" t="n"/>
+      <c r="AM8" s="7" t="n"/>
+      <c r="AN8" s="7" t="n"/>
+      <c r="AO8" s="7" t="n"/>
+      <c r="AP8" s="7" t="n"/>
+      <c r="AQ8" s="7" t="n"/>
+      <c r="AR8" s="7" t="n"/>
+      <c r="AS8" s="7" t="n"/>
+      <c r="AT8" s="7" t="n"/>
+      <c r="AU8" s="7" t="n"/>
+      <c r="AV8" s="7" t="n"/>
+      <c r="AW8" s="7" t="n"/>
+      <c r="AX8" s="7" t="n"/>
+      <c r="AY8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>11:42</t>
+        </is>
+      </c>
+      <c r="D9" s="5">
+        <f>IFERROR(C9/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="F9" s="5">
+        <f>IFERROR(E9/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="H9" t="n">
+        <v>16</v>
+      </c>
+      <c r="I9" t="n">
+        <v>2.8629</v>
+      </c>
+      <c r="J9" t="n">
+        <v>7</v>
+      </c>
+      <c r="K9" t="n">
+        <v>70</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>10</v>
+      </c>
+      <c r="R9" t="n">
+        <v>6</v>
+      </c>
+      <c r="S9" t="n">
+        <v>20</v>
+      </c>
+      <c r="T9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="U9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="V9" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="X9" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW9" t="inlineStr">
+        <is>
+          <t>2026-10-13 11:42:47.094626</t>
+        </is>
+      </c>
+      <c r="AX9" t="inlineStr">
+        <is>
+          <t>C:\Ugurcan\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Stage1\setups\Stage1\sessions\20261013-114246\20261013-114246.csv</t>
+        </is>
+      </c>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>C:\Ugurcan\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Stage1\setups\Stage1\sessions\20261013-114246\20261013-114246_struct.mat</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="D10" s="5">
+        <f>IFERROR(C10/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="F10" s="5">
+        <f>IFERROR(E10/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>7</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="U10" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="V10" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW10" t="inlineStr">
+        <is>
+          <t>2026-10-13 11:45:19.843221</t>
+        </is>
+      </c>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>C:\Ugurcan\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Stage1\setups\Stage1\sessions\20261013-114519\20261013-114519.csv</t>
+        </is>
+      </c>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>C:\Ugurcan\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Stage1\setups\Stage1\sessions\20261013-114519\20261013-114519_struct.mat</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n"/>
+      <c r="C11" s="9" t="n"/>
+      <c r="D11" s="9" t="n"/>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="9" t="n"/>
+      <c r="G11" s="9" t="n"/>
+      <c r="H11" s="9" t="n"/>
+      <c r="I11" s="9" t="n"/>
+      <c r="J11" s="9" t="n"/>
+      <c r="K11" s="9" t="n"/>
+      <c r="L11" s="9" t="n"/>
+      <c r="M11" s="9" t="n"/>
+      <c r="N11" s="9" t="n"/>
+      <c r="O11" s="9" t="n"/>
+      <c r="P11" s="9" t="n"/>
+      <c r="Q11" s="9" t="n"/>
+      <c r="R11" s="9" t="n"/>
+      <c r="S11" s="9" t="n"/>
+      <c r="T11" s="9" t="n"/>
+      <c r="U11" s="9" t="n"/>
+      <c r="V11" s="9" t="n"/>
+      <c r="W11" s="9" t="n"/>
+      <c r="X11" s="9" t="n"/>
+      <c r="Y11" s="9" t="n"/>
+      <c r="Z11" s="9" t="n"/>
+      <c r="AA11" s="9" t="n"/>
+      <c r="AB11" s="9" t="n"/>
+      <c r="AC11" s="9" t="n"/>
+      <c r="AD11" s="9" t="n"/>
+      <c r="AE11" s="9" t="n"/>
+      <c r="AF11" s="9" t="n"/>
+      <c r="AG11" s="9" t="n"/>
+      <c r="AH11" s="9" t="n"/>
+      <c r="AI11" s="9" t="n"/>
+      <c r="AJ11" s="9" t="n"/>
+      <c r="AK11" s="9" t="n"/>
+      <c r="AL11" s="9" t="n"/>
+      <c r="AM11" s="9" t="n"/>
+      <c r="AN11" s="9" t="n"/>
+      <c r="AO11" s="9" t="n"/>
+      <c r="AP11" s="9" t="n"/>
+      <c r="AQ11" s="9" t="n"/>
+      <c r="AR11" s="9" t="n"/>
+      <c r="AS11" s="9" t="n"/>
+      <c r="AT11" s="9" t="n"/>
+      <c r="AU11" s="9" t="n"/>
+      <c r="AV11" s="9" t="n"/>
+      <c r="AW11" s="9" t="n"/>
+      <c r="AX11" s="9" t="n"/>
+      <c r="AY11" s="9" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="D12" s="5">
+        <f>IFERROR(C12/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="F12" s="5">
+        <f>IFERROR(E12/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="H12" t="n">
+        <v>20</v>
+      </c>
+      <c r="I12" t="n">
+        <v>10.4954</v>
+      </c>
+      <c r="J12" t="n">
+        <v>7</v>
+      </c>
+      <c r="K12" t="n">
+        <v>98</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>8</v>
+      </c>
+      <c r="R12" t="n">
+        <v>11</v>
+      </c>
+      <c r="S12" t="n">
+        <v>24</v>
+      </c>
+      <c r="T12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="U12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="V12" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>0.5789473684210527</v>
+      </c>
+      <c r="Z12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW12" t="inlineStr">
+        <is>
+          <t>2026-10-13 11:44:01.488979</t>
+        </is>
+      </c>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>C:\Ugurcan\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Stage2\setups\Stage2\sessions\20261013-114400\20261013-114400.csv</t>
+        </is>
+      </c>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>C:\Ugurcan\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Stage2\setups\Stage2\sessions\20261013-114400\20261013-114400_struct.mat</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="13" t="n"/>
+      <c r="E13" s="13" t="n"/>
+      <c r="F13" s="13" t="n"/>
+      <c r="G13" s="13" t="n"/>
+      <c r="H13" s="13" t="n"/>
+      <c r="I13" s="13" t="n"/>
+      <c r="J13" s="13" t="n"/>
+      <c r="K13" s="13" t="n"/>
+      <c r="L13" s="13" t="n"/>
+      <c r="M13" s="13" t="n"/>
+      <c r="N13" s="13" t="n"/>
+      <c r="O13" s="13" t="n"/>
+      <c r="P13" s="13" t="n"/>
+      <c r="Q13" s="13" t="n"/>
+      <c r="R13" s="13" t="n"/>
+      <c r="S13" s="13" t="n"/>
+      <c r="T13" s="13" t="n"/>
+      <c r="U13" s="13" t="n"/>
+      <c r="V13" s="13" t="n"/>
+      <c r="W13" s="13" t="n"/>
+      <c r="X13" s="13" t="n"/>
+      <c r="Y13" s="13" t="n"/>
+      <c r="Z13" s="13" t="n"/>
+      <c r="AA13" s="13" t="n"/>
+      <c r="AB13" s="13" t="n"/>
+      <c r="AC13" s="13" t="n"/>
+      <c r="AD13" s="13" t="n"/>
+      <c r="AE13" s="13" t="n"/>
+      <c r="AF13" s="13" t="n"/>
+      <c r="AG13" s="13" t="n"/>
+      <c r="AH13" s="13" t="n"/>
+      <c r="AI13" s="13" t="n"/>
+      <c r="AJ13" s="13" t="n"/>
+      <c r="AK13" s="13" t="n"/>
+      <c r="AL13" s="13" t="n"/>
+      <c r="AM13" s="13" t="n"/>
+      <c r="AN13" s="13" t="n"/>
+      <c r="AO13" s="13" t="n"/>
+      <c r="AP13" s="13" t="n"/>
+      <c r="AQ13" s="13" t="n"/>
+      <c r="AR13" s="13" t="n"/>
+      <c r="AS13" s="13" t="n"/>
+      <c r="AT13" s="13" t="n"/>
+      <c r="AU13" s="13" t="n"/>
+      <c r="AV13" s="13" t="n"/>
+      <c r="AW13" s="13" t="n"/>
+      <c r="AX13" s="13" t="n"/>
+      <c r="AY13" s="13" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="D14" s="5">
+        <f>IFERROR(C14/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="5">
+        <f>IFERROR(E14/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="G14" t="b">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>35</v>
+      </c>
+      <c r="I14" t="n">
+        <v>7.895900000000001</v>
+      </c>
+      <c r="J14" t="n">
+        <v>7</v>
+      </c>
+      <c r="K14" t="n">
+        <v>105</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" t="n">
+        <v>1</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>1</v>
+      </c>
+      <c r="R14" t="n">
+        <v>16</v>
+      </c>
+      <c r="S14" t="n">
+        <v>18</v>
+      </c>
+      <c r="W14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Z14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF14" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>17</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ14" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AR14" t="n">
+        <v>70</v>
+      </c>
+      <c r="AS14" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>10000</v>
+      </c>
+      <c r="AW14" t="inlineStr">
+        <is>
+          <t>2026-10-13 11:45:30.059502</t>
+        </is>
+      </c>
+      <c r="AX14" t="inlineStr">
+        <is>
+          <t>C:\Ugurcan\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Stage3\setups\Stage3\sessions\20261013-114528\20261013-114528.csv</t>
+        </is>
+      </c>
+      <c r="AY14" t="inlineStr">
+        <is>
+          <t>C:\Ugurcan\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Stage3\setups\Stage3\sessions\20261013-114528\20261013-114528_struct.mat</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update training data from TRAINING03
</commit_message>
<xml_diff>
--- a/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
+++ b/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
@@ -2,30 +2,45 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible" windowHeight="9375" windowWidth="23160" xWindow="0" yWindow="0"/>
   </bookViews>
   <sheets>
     <sheet name="UM001" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="test_stage1" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="162913" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt formatCode="0.0%" numFmtId="164"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -39,7 +54,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -48,22 +63,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
+        <fgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2F0D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -77,30 +82,31 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="13">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="164" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="2" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="3" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="3" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle builtinId="0" name="Normal" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium9"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -461,63 +467,63 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY9"/>
+  <dimension ref="A1:AY12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
-    <col width="14" customWidth="1" min="25" max="25"/>
-    <col width="14" customWidth="1" min="26" max="26"/>
-    <col width="14" customWidth="1" min="27" max="27"/>
-    <col width="14" customWidth="1" min="28" max="28"/>
-    <col width="14" customWidth="1" min="29" max="29"/>
-    <col width="14" customWidth="1" min="30" max="30"/>
-    <col width="14" customWidth="1" min="31" max="31"/>
-    <col width="14" customWidth="1" min="32" max="32"/>
-    <col width="14" customWidth="1" min="33" max="33"/>
-    <col width="14" customWidth="1" min="34" max="34"/>
-    <col width="14" customWidth="1" min="35" max="35"/>
-    <col width="14" customWidth="1" min="36" max="36"/>
-    <col width="14" customWidth="1" min="37" max="37"/>
-    <col width="14" customWidth="1" min="38" max="38"/>
-    <col width="14" customWidth="1" min="39" max="39"/>
-    <col width="14" customWidth="1" min="40" max="40"/>
-    <col width="14" customWidth="1" min="41" max="41"/>
-    <col width="14" customWidth="1" min="42" max="42"/>
-    <col width="14" customWidth="1" min="43" max="43"/>
-    <col width="14" customWidth="1" min="44" max="44"/>
-    <col width="14" customWidth="1" min="45" max="45"/>
-    <col width="14" customWidth="1" min="46" max="46"/>
-    <col width="14" customWidth="1" min="47" max="47"/>
-    <col width="14" customWidth="1" min="48" max="48"/>
-    <col hidden="1" width="14" customWidth="1" min="49" max="49"/>
-    <col width="14" customWidth="1" min="50" max="50"/>
-    <col width="14" customWidth="1" min="51" max="51"/>
+    <col customWidth="1" max="48" min="1" width="14"/>
+    <col customWidth="1" max="2" min="2" width="14"/>
+    <col customWidth="1" max="3" min="3" width="14"/>
+    <col customWidth="1" max="4" min="4" width="14"/>
+    <col customWidth="1" max="5" min="5" width="14"/>
+    <col customWidth="1" max="6" min="6" width="14"/>
+    <col customWidth="1" max="7" min="7" width="14"/>
+    <col customWidth="1" max="8" min="8" width="14"/>
+    <col customWidth="1" max="9" min="9" width="14"/>
+    <col customWidth="1" max="10" min="10" width="14"/>
+    <col customWidth="1" max="11" min="11" width="14"/>
+    <col customWidth="1" max="12" min="12" width="14"/>
+    <col customWidth="1" max="13" min="13" width="14"/>
+    <col customWidth="1" max="14" min="14" width="14"/>
+    <col customWidth="1" max="15" min="15" width="14"/>
+    <col customWidth="1" max="16" min="16" width="14"/>
+    <col customWidth="1" max="17" min="17" width="14"/>
+    <col customWidth="1" max="18" min="18" width="14"/>
+    <col customWidth="1" max="19" min="19" width="14"/>
+    <col customWidth="1" max="20" min="20" width="14"/>
+    <col customWidth="1" max="21" min="21" width="14"/>
+    <col customWidth="1" max="22" min="22" width="14"/>
+    <col customWidth="1" max="23" min="23" width="14"/>
+    <col customWidth="1" max="24" min="24" width="14"/>
+    <col customWidth="1" max="25" min="25" width="14"/>
+    <col customWidth="1" max="26" min="26" width="14"/>
+    <col customWidth="1" max="27" min="27" width="14"/>
+    <col customWidth="1" max="28" min="28" width="14"/>
+    <col customWidth="1" max="29" min="29" width="14"/>
+    <col customWidth="1" max="30" min="30" width="14"/>
+    <col customWidth="1" max="31" min="31" width="14"/>
+    <col customWidth="1" max="32" min="32" width="14"/>
+    <col customWidth="1" max="33" min="33" width="14"/>
+    <col customWidth="1" max="34" min="34" width="14"/>
+    <col customWidth="1" max="35" min="35" width="14"/>
+    <col customWidth="1" max="36" min="36" width="14"/>
+    <col customWidth="1" max="37" min="37" width="14"/>
+    <col customWidth="1" max="38" min="38" width="14"/>
+    <col customWidth="1" max="39" min="39" width="14"/>
+    <col customWidth="1" max="40" min="40" width="14"/>
+    <col customWidth="1" max="41" min="41" width="14"/>
+    <col customWidth="1" max="42" min="42" width="14"/>
+    <col customWidth="1" max="43" min="43" width="14"/>
+    <col customWidth="1" max="44" min="44" width="14"/>
+    <col customWidth="1" max="45" min="45" width="14"/>
+    <col customWidth="1" max="46" min="46" width="14"/>
+    <col customWidth="1" max="47" min="47" width="14"/>
+    <col customWidth="1" max="48" min="48" width="14"/>
+    <col customWidth="1" hidden="1" max="49" min="49" width="14"/>
+    <col customWidth="1" max="51" min="50" width="14"/>
+    <col customWidth="1" max="51" min="51" width="14"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row customHeight="1" ht="15.75" r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Animal: UM001</t>
@@ -572,319 +578,319 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+    <row customHeight="1" ht="45" r="7">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Time (HH:MM)</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Weight (g)</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>Weight %</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>Weight after task (g)</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="10" t="inlineStr">
         <is>
           <t>Weight after task %</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="10" t="inlineStr">
         <is>
           <t>Water given by hand after task</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" s="10" t="inlineStr">
         <is>
           <t>Trials</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I7" s="10" t="inlineStr">
         <is>
           <t>Duration (s)</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="J7" s="10" t="inlineStr">
         <is>
           <t>Reward Amount (uL)</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K7" s="10" t="inlineStr">
         <is>
           <t>Total Volume (uL)</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="L7" s="10" t="inlineStr">
         <is>
           <t>Aborts</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="M7" s="10" t="inlineStr">
         <is>
           <t>Withheld</t>
         </is>
       </c>
-      <c r="N7" s="3" t="inlineStr">
+      <c r="N7" s="10" t="inlineStr">
         <is>
           <t>No-movement</t>
         </is>
       </c>
-      <c r="O7" s="3" t="inlineStr">
+      <c r="O7" s="10" t="inlineStr">
         <is>
           <t>Incorrect</t>
         </is>
       </c>
-      <c r="P7" s="3" t="inlineStr">
+      <c r="P7" s="10" t="inlineStr">
         <is>
           <t>Wheel Aborts</t>
         </is>
       </c>
-      <c r="Q7" s="3" t="inlineStr">
+      <c r="Q7" s="10" t="inlineStr">
         <is>
           <t>L turns</t>
         </is>
       </c>
-      <c r="R7" s="3" t="inlineStr">
+      <c r="R7" s="10" t="inlineStr">
         <is>
           <t>R turns</t>
         </is>
       </c>
-      <c r="S7" s="3" t="inlineStr">
+      <c r="S7" s="10" t="inlineStr">
         <is>
           <t>Licks</t>
         </is>
       </c>
-      <c r="T7" s="3" t="inlineStr">
+      <c r="T7" s="10" t="inlineStr">
         <is>
           <t>Threshold start (deg)</t>
         </is>
       </c>
-      <c r="U7" s="3" t="inlineStr">
+      <c r="U7" s="10" t="inlineStr">
         <is>
           <t>Threshold end (deg)</t>
         </is>
       </c>
-      <c r="V7" s="3" t="inlineStr">
+      <c r="V7" s="10" t="inlineStr">
         <is>
           <t>Threshold end (% final)</t>
         </is>
       </c>
-      <c r="W7" s="3" t="inlineStr">
+      <c r="W7" s="10" t="inlineStr">
         <is>
           <t>ITI (s)</t>
         </is>
       </c>
-      <c r="X7" s="3" t="inlineStr">
+      <c r="X7" s="10" t="inlineStr">
         <is>
           <t>Gain mult (Stage 1)</t>
         </is>
       </c>
-      <c r="Y7" s="3" t="inlineStr">
+      <c r="Y7" s="10" t="inlineStr">
         <is>
           <t>Direction ratio (Stage 2)</t>
         </is>
       </c>
-      <c r="Z7" s="3" t="inlineStr">
+      <c r="Z7" s="10" t="inlineStr">
         <is>
           <t>Simple gates met</t>
         </is>
       </c>
-      <c r="AA7" s="3" t="inlineStr">
+      <c r="AA7" s="10" t="inlineStr">
         <is>
           <t>Response Thresh Start (deg)</t>
         </is>
       </c>
-      <c r="AB7" s="3" t="inlineStr">
+      <c r="AB7" s="10" t="inlineStr">
         <is>
           <t>Response Thresh End (deg)</t>
         </is>
       </c>
-      <c r="AC7" s="3" t="inlineStr">
+      <c r="AC7" s="10" t="inlineStr">
         <is>
           <t>Quiescence Start (s)</t>
         </is>
       </c>
-      <c r="AD7" s="3" t="inlineStr">
+      <c r="AD7" s="10" t="inlineStr">
         <is>
           <t>Quiescence End (s)</t>
         </is>
       </c>
-      <c r="AE7" s="3" t="inlineStr">
+      <c r="AE7" s="10" t="inlineStr">
         <is>
           <t>In-trial Threshold (deg)</t>
         </is>
       </c>
-      <c r="AF7" s="3" t="inlineStr">
+      <c r="AF7" s="10" t="inlineStr">
         <is>
           <t>Click Attenuated (Stage 4)</t>
         </is>
       </c>
-      <c r="AG7" s="3" t="inlineStr">
+      <c r="AG7" s="10" t="inlineStr">
         <is>
           <t>Accuracy (gamma=1.0)</t>
         </is>
       </c>
-      <c r="AH7" s="3" t="inlineStr">
+      <c r="AH7" s="10" t="inlineStr">
         <is>
           <t>Abort Rate</t>
         </is>
       </c>
-      <c r="AI7" s="3" t="inlineStr">
+      <c r="AI7" s="10" t="inlineStr">
         <is>
           <t>Aborts: Quiescence</t>
         </is>
       </c>
-      <c r="AJ7" s="3" t="inlineStr">
+      <c r="AJ7" s="10" t="inlineStr">
         <is>
           <t>Aborts: Cue</t>
         </is>
       </c>
-      <c r="AK7" s="3" t="inlineStr">
+      <c r="AK7" s="10" t="inlineStr">
         <is>
           <t>Aborts: Delay</t>
         </is>
       </c>
-      <c r="AL7" s="3" t="inlineStr">
+      <c r="AL7" s="10" t="inlineStr">
         <is>
           <t>Aborts: Response</t>
         </is>
       </c>
-      <c r="AM7" s="3" t="inlineStr">
+      <c r="AM7" s="10" t="inlineStr">
         <is>
           <t>Warmup Trials</t>
         </is>
       </c>
-      <c r="AN7" s="3" t="inlineStr">
+      <c r="AN7" s="10" t="inlineStr">
         <is>
           <t>Repeat Trials</t>
         </is>
       </c>
-      <c r="AO7" s="3" t="inlineStr">
+      <c r="AO7" s="10" t="inlineStr">
         <is>
           <t>Session Water (uL)</t>
         </is>
       </c>
-      <c r="AP7" s="3" t="inlineStr">
+      <c r="AP7" s="10" t="inlineStr">
         <is>
           <t>Staircase Advanced (Stage 5)</t>
         </is>
       </c>
-      <c r="AQ7" s="3" t="inlineStr">
+      <c r="AQ7" s="10" t="inlineStr">
         <is>
           <t>Git Commit</t>
         </is>
       </c>
-      <c r="AR7" s="3" t="inlineStr">
+      <c r="AR7" s="10" t="inlineStr">
         <is>
           <t>Target SPL (dB)</t>
         </is>
       </c>
-      <c r="AS7" s="3" t="inlineStr">
+      <c r="AS7" s="10" t="inlineStr">
         <is>
           <t>Left Freq (Hz)</t>
         </is>
       </c>
-      <c r="AT7" s="3" t="inlineStr">
+      <c r="AT7" s="10" t="inlineStr">
         <is>
           <t>Right Freq (Hz)</t>
         </is>
       </c>
-      <c r="AU7" s="3" t="inlineStr">
+      <c r="AU7" s="10" t="inlineStr">
         <is>
           <t>Num. Sessions</t>
         </is>
       </c>
-      <c r="AV7" s="3" t="inlineStr">
+      <c r="AV7" s="10" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="AW7" s="3" t="inlineStr">
+      <c r="AW7" s="10" t="inlineStr">
         <is>
           <t>Session started</t>
         </is>
       </c>
-      <c r="AX7" s="3" t="inlineStr">
+      <c r="AX7" s="10" t="inlineStr">
         <is>
           <t>Session data (local path)</t>
         </is>
       </c>
-      <c r="AY7" s="3" t="inlineStr">
+      <c r="AY7" s="10" t="inlineStr">
         <is>
           <t>Session struct (local path)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Stage 1</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="7" t="n"/>
-      <c r="H8" s="7" t="n"/>
-      <c r="I8" s="7" t="n"/>
-      <c r="J8" s="7" t="n"/>
-      <c r="K8" s="7" t="n"/>
-      <c r="L8" s="7" t="n"/>
-      <c r="M8" s="7" t="n"/>
-      <c r="N8" s="7" t="n"/>
-      <c r="O8" s="7" t="n"/>
-      <c r="P8" s="7" t="n"/>
-      <c r="Q8" s="7" t="n"/>
-      <c r="R8" s="7" t="n"/>
-      <c r="S8" s="7" t="n"/>
-      <c r="T8" s="7" t="n"/>
-      <c r="U8" s="7" t="n"/>
-      <c r="V8" s="7" t="n"/>
-      <c r="W8" s="7" t="n"/>
-      <c r="X8" s="7" t="n"/>
-      <c r="Y8" s="7" t="n"/>
-      <c r="Z8" s="7" t="n"/>
-      <c r="AA8" s="7" t="n"/>
-      <c r="AB8" s="7" t="n"/>
-      <c r="AC8" s="7" t="n"/>
-      <c r="AD8" s="7" t="n"/>
-      <c r="AE8" s="7" t="n"/>
-      <c r="AF8" s="7" t="n"/>
-      <c r="AG8" s="7" t="n"/>
-      <c r="AH8" s="7" t="n"/>
-      <c r="AI8" s="7" t="n"/>
-      <c r="AJ8" s="7" t="n"/>
-      <c r="AK8" s="7" t="n"/>
-      <c r="AL8" s="7" t="n"/>
-      <c r="AM8" s="7" t="n"/>
-      <c r="AN8" s="7" t="n"/>
-      <c r="AO8" s="7" t="n"/>
-      <c r="AP8" s="7" t="n"/>
-      <c r="AQ8" s="7" t="n"/>
-      <c r="AR8" s="7" t="n"/>
-      <c r="AS8" s="7" t="n"/>
-      <c r="AT8" s="7" t="n"/>
-      <c r="AU8" s="7" t="n"/>
-      <c r="AV8" s="7" t="n"/>
-      <c r="AW8" s="7" t="n"/>
-      <c r="AX8" s="7" t="n"/>
-      <c r="AY8" s="7" t="n"/>
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="12" t="n"/>
+      <c r="E8" s="12" t="n"/>
+      <c r="F8" s="12" t="n"/>
+      <c r="G8" s="12" t="n"/>
+      <c r="H8" s="12" t="n"/>
+      <c r="I8" s="12" t="n"/>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="12" t="n"/>
+      <c r="L8" s="12" t="n"/>
+      <c r="M8" s="12" t="n"/>
+      <c r="N8" s="12" t="n"/>
+      <c r="O8" s="12" t="n"/>
+      <c r="P8" s="12" t="n"/>
+      <c r="Q8" s="12" t="n"/>
+      <c r="R8" s="12" t="n"/>
+      <c r="S8" s="12" t="n"/>
+      <c r="T8" s="12" t="n"/>
+      <c r="U8" s="12" t="n"/>
+      <c r="V8" s="12" t="n"/>
+      <c r="W8" s="12" t="n"/>
+      <c r="X8" s="12" t="n"/>
+      <c r="Y8" s="12" t="n"/>
+      <c r="Z8" s="12" t="n"/>
+      <c r="AA8" s="12" t="n"/>
+      <c r="AB8" s="12" t="n"/>
+      <c r="AC8" s="12" t="n"/>
+      <c r="AD8" s="12" t="n"/>
+      <c r="AE8" s="12" t="n"/>
+      <c r="AF8" s="12" t="n"/>
+      <c r="AG8" s="12" t="n"/>
+      <c r="AH8" s="12" t="n"/>
+      <c r="AI8" s="12" t="n"/>
+      <c r="AJ8" s="12" t="n"/>
+      <c r="AK8" s="12" t="n"/>
+      <c r="AL8" s="12" t="n"/>
+      <c r="AM8" s="12" t="n"/>
+      <c r="AN8" s="12" t="n"/>
+      <c r="AO8" s="12" t="n"/>
+      <c r="AP8" s="12" t="n"/>
+      <c r="AQ8" s="12" t="n"/>
+      <c r="AR8" s="12" t="n"/>
+      <c r="AS8" s="12" t="n"/>
+      <c r="AT8" s="12" t="n"/>
+      <c r="AU8" s="12" t="n"/>
+      <c r="AV8" s="12" t="n"/>
+      <c r="AW8" s="12" t="n"/>
+      <c r="AX8" s="12" t="n"/>
+      <c r="AY8" s="12" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -942,10 +948,10 @@
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="R9" t="n">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="S9" t="n">
         <v>160</v>
@@ -1007,7 +1013,404 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>13:57</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D10" s="5">
+        <f>IFERROR(C10/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="E10" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F10" s="5">
+        <f>IFERROR(E10/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="G10" t="b">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>62</v>
+      </c>
+      <c r="I10" t="n">
+        <v>10.4986</v>
+      </c>
+      <c r="J10" t="n">
+        <v>10</v>
+      </c>
+      <c r="K10" t="n">
+        <v>460</v>
+      </c>
+      <c r="L10" t="n">
+        <v>387</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="n">
+        <v>10</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>22</v>
+      </c>
+      <c r="R10" t="n">
+        <v>30</v>
+      </c>
+      <c r="S10" t="n">
+        <v>527</v>
+      </c>
+      <c r="T10" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="U10" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="V10" s="4" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0.4999999999999999</v>
+      </c>
+      <c r="X10" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="AH10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW10" t="inlineStr">
+        <is>
+          <t>2026-10-22 13:57:06.324806</t>
+        </is>
+      </c>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>C:\Ugurcan\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Stage1\setups\Stage1\sessions\20261022-135705\20261022-135705.csv</t>
+        </is>
+      </c>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>C:\Ugurcan\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Stage1\setups\Stage1\sessions\20261022-135705\20261022-135705_struct.mat</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>14:02</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>24</v>
+      </c>
+      <c r="D11" s="5">
+        <f>IFERROR(C11/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="E11" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="F11" s="5">
+        <f>IFERROR(E11/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="G11" t="b">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>191</v>
+      </c>
+      <c r="I11" t="n">
+        <v>10.4999</v>
+      </c>
+      <c r="J11" t="n">
+        <v>10</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1170</v>
+      </c>
+      <c r="L11" t="n">
+        <v>366</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>41</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>59</v>
+      </c>
+      <c r="R11" t="n">
+        <v>91</v>
+      </c>
+      <c r="S11" t="n">
+        <v>1909</v>
+      </c>
+      <c r="T11" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="U11" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="V11" s="4" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="X11" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="AH11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW11" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:02:22.920559</t>
+        </is>
+      </c>
+      <c r="AX11" t="inlineStr">
+        <is>
+          <t>C:\Ugurcan\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Stage1\setups\Stage1\sessions\20261022-140221\20261022-140221.csv</t>
+        </is>
+      </c>
+      <c r="AY11" t="inlineStr">
+        <is>
+          <t>C:\Ugurcan\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Stage1\setups\Stage1\sessions\20261022-140221\20261022-140221_struct.mat</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>10:28</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="D12" s="5">
+        <f>IFERROR(C12/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="E12" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="F12" s="5">
+        <f>IFERROR(E12/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="G12" t="b">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>221</v>
+      </c>
+      <c r="I12" t="n">
+        <v>11.7722</v>
+      </c>
+      <c r="J12" t="n">
+        <v>7</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1470</v>
+      </c>
+      <c r="L12" t="n">
+        <v>103</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="n">
+        <v>6</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>111</v>
+      </c>
+      <c r="R12" t="n">
+        <v>104</v>
+      </c>
+      <c r="S12" t="n">
+        <v>2131</v>
+      </c>
+      <c r="T12" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="U12" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="V12" s="4" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="X12" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="AH12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW12" t="inlineStr">
+        <is>
+          <t>2026-10-27 10:28:44.823299</t>
+        </is>
+      </c>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>C:\Ugurcan\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Stage1\setups\Stage1\sessions\20261027-102843\20261027-102843.csv</t>
+        </is>
+      </c>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>C:\Ugurcan\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Stage1\setups\Stage1\sessions\20261027-102843\20261027-102843_struct.mat</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Animal: test_stage1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>DOB</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Sex</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Strain</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Baseline weight (g)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Run on stock pybpod-api; QC follow-ups for 20261027-102843
- Fix "submodule points to a commit that doesn't exist" on other boxes: pybpod now
  pins pybpod-api to the official v1.8.2 (4c9ced5). install_session_lock() installs
  the locked add_message(msg, flush) itself, so the stages work on stock pybpod-api;
  the offline suite passes against both.
- Audit: detrend the wheel clock-map check (11 ms -> 0.41 ms around 21.5 ppm drift);
  reader-stall check skips trial 1 and names trials over budget.
- Keepalive WHEEL_POS module times can no longer step backward.
- Parser: TRIAL_INIT_START filed under its own trial; wheel rows before trial 1 kept.
- Lick chatter (In < 40 ms after the previous Out) merged for derived lick counts and
  dashboard rasters; raw rows untouched.
- Training log and UM001 audit report refreshed; validation Section 19 added.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
+++ b/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
@@ -964,7 +964,7 @@
         <v>70</v>
       </c>
       <c r="T9" t="n">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="U9" t="n">
         <v>3.5</v>
@@ -1088,7 +1088,7 @@
         <v>30</v>
       </c>
       <c r="T10" t="n">
-        <v>527</v>
+        <v>247</v>
       </c>
       <c r="U10" t="n">
         <v>4.2</v>
@@ -1207,7 +1207,7 @@
         <v>91</v>
       </c>
       <c r="T11" t="n">
-        <v>1909</v>
+        <v>600</v>
       </c>
       <c r="U11" t="n">
         <v>4.2</v>
@@ -1326,7 +1326,7 @@
         <v>104</v>
       </c>
       <c r="T12" t="n">
-        <v>2131</v>
+        <v>1757</v>
       </c>
       <c r="U12" t="n">
         <v>4.9</v>

</xml_diff>

<commit_message>
Daily water cap per animal, trial cap 250, fix training-log Duration
- Stage 1/2: water capped at 1.5 mL consumed per animal per calendar day across all of
  its sessions (session_csv_parser.water_consumed_today()); a session started with the
  day's water used up ends before trial 1 and doesn't enter the advancement history.
  Dashboard warns before launching one. Stage 1 trial cap back to 250 per session.
- Training log Duration was max-min of trial-relative event times (~one trial); now
  first trial start -> last trial end on the Bpod clock. Rebuilt training_log.xlsx.
- Audit coverage check excludes normal machine-to-machine handovers (requires 99% of
  the rest); fast 1.2 s trials no longer fail it, the old hold-wait design still does.
- UM001 20261028 sessions' audit reports; validation Section 20.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
+++ b/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
@@ -931,7 +931,7 @@
         <v>214</v>
       </c>
       <c r="I9" t="n">
-        <v>10.4995</v>
+        <v>1269.200002</v>
       </c>
       <c r="J9" t="n">
         <v>7</v>
@@ -1055,7 +1055,7 @@
         <v>62</v>
       </c>
       <c r="I10" t="n">
-        <v>10.4986</v>
+        <v>225.758103</v>
       </c>
       <c r="J10" t="n">
         <v>10</v>
@@ -1174,7 +1174,7 @@
         <v>191</v>
       </c>
       <c r="I11" t="n">
-        <v>10.4999</v>
+        <v>927.9607020000001</v>
       </c>
       <c r="J11" t="n">
         <v>10</v>
@@ -1293,7 +1293,7 @@
         <v>221</v>
       </c>
       <c r="I12" t="n">
-        <v>11.7722</v>
+        <v>573.3331030000001</v>
       </c>
       <c r="J12" t="n">
         <v>7</v>
@@ -1412,7 +1412,7 @@
         <v>303</v>
       </c>
       <c r="I13" t="n">
-        <v>16.4147</v>
+        <v>454.989606</v>
       </c>
       <c r="J13" t="n">
         <v>7</v>

</xml_diff>

<commit_message>
Training log: Duration in minutes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
+++ b/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
@@ -622,7 +622,7 @@
       </c>
       <c r="I7" s="10" t="inlineStr">
         <is>
-          <t>Duration (s)</t>
+          <t>Duration (min)</t>
         </is>
       </c>
       <c r="J7" s="10" t="inlineStr">
@@ -931,7 +931,7 @@
         <v>214</v>
       </c>
       <c r="I9" t="n">
-        <v>1269.200002</v>
+        <v>21.2</v>
       </c>
       <c r="J9" t="n">
         <v>7</v>
@@ -1055,7 +1055,7 @@
         <v>62</v>
       </c>
       <c r="I10" t="n">
-        <v>225.758103</v>
+        <v>3.8</v>
       </c>
       <c r="J10" t="n">
         <v>10</v>
@@ -1174,7 +1174,7 @@
         <v>191</v>
       </c>
       <c r="I11" t="n">
-        <v>927.9607020000001</v>
+        <v>15.5</v>
       </c>
       <c r="J11" t="n">
         <v>10</v>
@@ -1293,7 +1293,7 @@
         <v>221</v>
       </c>
       <c r="I12" t="n">
-        <v>573.3331030000001</v>
+        <v>9.6</v>
       </c>
       <c r="J12" t="n">
         <v>7</v>
@@ -1412,7 +1412,7 @@
         <v>303</v>
       </c>
       <c r="I13" t="n">
-        <v>454.989606</v>
+        <v>7.6</v>
       </c>
       <c r="J13" t="n">
         <v>7</v>

</xml_diff>

<commit_message>
Session data: UM001 20261029-144232 (Stage 1, water cap), training log
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
+++ b/_projects/AuditoryEvidenceAccum/records/training_log.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ13"/>
+  <dimension ref="A1:AZ14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col customWidth="1" max="48" min="1" width="14"/>
@@ -1502,6 +1502,116 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>14:42</t>
+        </is>
+      </c>
+      <c r="D14" s="5">
+        <f>IFERROR(C14/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="5">
+        <f>IFERROR(E14/$B$5,"")</f>
+        <v/>
+      </c>
+      <c r="H14" t="n">
+        <v>215</v>
+      </c>
+      <c r="I14" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="J14" t="n">
+        <v>7</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1505</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1505</v>
+      </c>
+      <c r="M14" t="n">
+        <v>104</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" t="n">
+        <v>112</v>
+      </c>
+      <c r="S14" t="n">
+        <v>103</v>
+      </c>
+      <c r="T14" t="n">
+        <v>2056</v>
+      </c>
+      <c r="U14" t="n">
+        <v>6.999999999999999</v>
+      </c>
+      <c r="V14" t="n">
+        <v>6.999999999999999</v>
+      </c>
+      <c r="W14" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="AI14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX14" t="inlineStr">
+        <is>
+          <t>2026-10-29 14:42:34.495925</t>
+        </is>
+      </c>
+      <c r="AY14" t="inlineStr">
+        <is>
+          <t>C:\Ugurcan\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Stage1\setups\Stage1\sessions\20261029-144232\20261029-144232.csv</t>
+        </is>
+      </c>
+      <c r="AZ14" t="inlineStr">
+        <is>
+          <t>C:\Ugurcan\Experimental-Tasks\_projects\AuditoryEvidenceAccum\experiments\Stage1\setups\Stage1\sessions\20261029-144232\20261029-144232_struct.mat</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>

</xml_diff>